<commit_message>
chore: actualizar precios 4 tiendas [automatico]
</commit_message>
<xml_diff>
--- a/GAMES LIST - AUTO.xlsx
+++ b/GAMES LIST - AUTO.xlsx
@@ -925,16 +925,16 @@
         <v>15</v>
       </c>
       <c r="D12">
-        <v>87338</v>
+        <v>87322</v>
       </c>
       <c r="E12">
         <v>82201</v>
       </c>
       <c r="F12">
-        <v>102338</v>
+        <v>102322</v>
       </c>
       <c r="G12">
-        <v>147367</v>
+        <v>147344</v>
       </c>
       <c r="H12">
         <v>15000</v>
@@ -1799,16 +1799,16 @@
         <v>15</v>
       </c>
       <c r="D32">
-        <v>77472</v>
+        <v>77348</v>
       </c>
       <c r="E32">
         <v>109608</v>
       </c>
       <c r="F32">
-        <v>92472</v>
+        <v>92348</v>
       </c>
       <c r="G32">
-        <v>133160</v>
+        <v>132981</v>
       </c>
       <c r="H32">
         <v>15000</v>
@@ -1979,16 +1979,16 @@
         <v>15</v>
       </c>
       <c r="D36">
-        <v>47017</v>
+        <v>46939</v>
       </c>
       <c r="E36">
         <v>127879</v>
       </c>
       <c r="F36">
-        <v>74017</v>
+        <v>73939</v>
       </c>
       <c r="G36">
-        <v>106584</v>
+        <v>106472</v>
       </c>
       <c r="H36">
         <v>27000</v>
@@ -2587,16 +2587,16 @@
         <v>15</v>
       </c>
       <c r="D50">
-        <v>37433</v>
+        <v>37355</v>
       </c>
       <c r="E50">
         <v>63930</v>
       </c>
       <c r="F50">
-        <v>52433</v>
+        <v>52355</v>
       </c>
       <c r="G50">
-        <v>75504</v>
+        <v>75391</v>
       </c>
       <c r="H50">
         <v>15000</v>
@@ -2947,16 +2947,16 @@
         <v>15</v>
       </c>
       <c r="D58">
-        <v>21136</v>
+        <v>20886</v>
       </c>
       <c r="E58">
         <v>36524</v>
       </c>
       <c r="F58">
-        <v>36136</v>
+        <v>35886</v>
       </c>
       <c r="G58">
-        <v>52036</v>
+        <v>51676</v>
       </c>
       <c r="H58">
         <v>15000</v>
@@ -3036,19 +3036,19 @@
         <v>15</v>
       </c>
       <c r="D60">
-        <v>26365</v>
+        <v>0</v>
       </c>
       <c r="E60">
         <v>49313</v>
       </c>
       <c r="F60">
-        <v>41365</v>
+        <v>0</v>
       </c>
       <c r="G60">
-        <v>59566</v>
+        <v>0</v>
       </c>
       <c r="H60">
-        <v>15000</v>
+        <v>0</v>
       </c>
       <c r="I60" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/268910/Cuphead/?curator_clanid=4777282","Abrir Steam")</f>
@@ -3734,19 +3734,19 @@
         <v>15</v>
       </c>
       <c r="D76">
-        <v>86667</v>
+        <v>0</v>
       </c>
       <c r="E76">
         <v>127879</v>
       </c>
       <c r="F76">
-        <v>101667</v>
+        <v>0</v>
       </c>
       <c r="G76">
-        <v>146400</v>
+        <v>0</v>
       </c>
       <c r="H76">
-        <v>15000</v>
+        <v>0</v>
       </c>
       <c r="I76" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/3280350/DEATH_STRANDING_2_ON_THE_BEACH/","Abrir Steam")</f>
@@ -4083,19 +4083,19 @@
         <v>15</v>
       </c>
       <c r="D84">
-        <v>0</v>
+        <v>47158</v>
       </c>
       <c r="E84">
         <v>102299</v>
       </c>
       <c r="F84">
-        <v>0</v>
+        <v>70898</v>
       </c>
       <c r="G84">
-        <v>0</v>
+        <v>102093</v>
       </c>
       <c r="H84">
-        <v>0</v>
+        <v>23740</v>
       </c>
       <c r="I84" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/1790600/DRAGON_BALL_Sparking_ZERO/","Abrir Steam")</f>
@@ -4258,19 +4258,19 @@
         <v>15</v>
       </c>
       <c r="D88">
-        <v>166418</v>
+        <v>0</v>
       </c>
       <c r="E88">
         <v>160767</v>
       </c>
       <c r="F88">
-        <v>181418</v>
+        <v>0</v>
       </c>
       <c r="G88">
-        <v>261242</v>
+        <v>0</v>
       </c>
       <c r="H88">
-        <v>15000</v>
+        <v>0</v>
       </c>
       <c r="I88" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/1790600/DRAGON_BALL_Sparking_ZERO/","Abrir Steam")</f>
@@ -4608,19 +4608,19 @@
         <v>15</v>
       </c>
       <c r="D96">
-        <v>61878</v>
+        <v>0</v>
       </c>
       <c r="E96">
         <v>82201</v>
       </c>
       <c r="F96">
-        <v>76878</v>
+        <v>0</v>
       </c>
       <c r="G96">
-        <v>110704</v>
+        <v>0</v>
       </c>
       <c r="H96">
-        <v>15000</v>
+        <v>0</v>
       </c>
       <c r="I96" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/3008130/Dying_Light_The_Beast/","Abrir Steam")</f>
@@ -4698,16 +4698,16 @@
         <v>15</v>
       </c>
       <c r="D98">
-        <v>76910</v>
+        <v>76676</v>
       </c>
       <c r="E98">
         <v>94991</v>
       </c>
       <c r="F98">
-        <v>91910</v>
+        <v>91676</v>
       </c>
       <c r="G98">
-        <v>132350</v>
+        <v>132013</v>
       </c>
       <c r="H98">
         <v>15000</v>
@@ -5483,19 +5483,19 @@
         <v>15</v>
       </c>
       <c r="D116">
-        <v>0</v>
+        <v>167417</v>
       </c>
       <c r="E116">
         <v>146150</v>
       </c>
       <c r="F116">
-        <v>0</v>
+        <v>182417</v>
       </c>
       <c r="G116">
-        <v>0</v>
+        <v>262680</v>
       </c>
       <c r="H116">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="I116" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/1245620/ELDEN_RING/","Abrir Steam")</f>
@@ -6530,19 +6530,19 @@
         <v>15</v>
       </c>
       <c r="D140">
-        <v>37667</v>
+        <v>37651</v>
       </c>
       <c r="E140">
         <v>91337</v>
       </c>
       <c r="F140">
-        <v>62169</v>
+        <v>62162</v>
       </c>
       <c r="G140">
-        <v>89523</v>
+        <v>89513</v>
       </c>
       <c r="H140">
-        <v>24502</v>
+        <v>24511</v>
       </c>
       <c r="I140" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/2215430/Ghost_of_Tsushima_VERSIN_DEL_DIRECTOR/?l=spanish","Abrir Steam")</f>
@@ -6618,19 +6618,19 @@
         <v>15</v>
       </c>
       <c r="D142">
-        <v>22853</v>
+        <v>0</v>
       </c>
       <c r="E142">
         <v>91337</v>
       </c>
       <c r="F142">
-        <v>49853</v>
+        <v>0</v>
       </c>
       <c r="G142">
-        <v>71788</v>
+        <v>0</v>
       </c>
       <c r="H142">
-        <v>27000</v>
+        <v>0</v>
       </c>
       <c r="I142" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/1593500/God_of_War/","Abrir Steam")</f>
@@ -6706,19 +6706,19 @@
         <v>15</v>
       </c>
       <c r="D144">
-        <v>44520</v>
+        <v>44379</v>
       </c>
       <c r="E144">
         <v>91337</v>
       </c>
       <c r="F144">
-        <v>64910</v>
+        <v>64853</v>
       </c>
       <c r="G144">
-        <v>93470</v>
+        <v>93388</v>
       </c>
       <c r="H144">
-        <v>20390</v>
+        <v>20474</v>
       </c>
       <c r="I144" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/2322010/God_of_War_Ragnark/?curator_clanid=4777282","Abrir Steam")</f>
@@ -6883,16 +6883,16 @@
         <v>15</v>
       </c>
       <c r="D148">
-        <v>36543</v>
+        <v>36527</v>
       </c>
       <c r="E148">
         <v>62103</v>
       </c>
       <c r="F148">
-        <v>51543</v>
+        <v>51527</v>
       </c>
       <c r="G148">
-        <v>74222</v>
+        <v>74199</v>
       </c>
       <c r="H148">
         <v>15000</v>
@@ -7855,16 +7855,16 @@
         <v>15</v>
       </c>
       <c r="D170">
-        <v>68981</v>
+        <v>68965</v>
       </c>
       <c r="E170">
         <v>109608</v>
       </c>
       <c r="F170">
-        <v>83981</v>
+        <v>83965</v>
       </c>
       <c r="G170">
-        <v>120933</v>
+        <v>120910</v>
       </c>
       <c r="H170">
         <v>15000</v>
@@ -8033,19 +8033,19 @@
         <v>15</v>
       </c>
       <c r="D174">
-        <v>48032</v>
+        <v>47845</v>
       </c>
       <c r="E174">
         <v>91337</v>
       </c>
       <c r="F174">
-        <v>66315</v>
+        <v>66240</v>
       </c>
       <c r="G174">
-        <v>95494</v>
+        <v>95386</v>
       </c>
       <c r="H174">
-        <v>18283</v>
+        <v>18395</v>
       </c>
       <c r="I174" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/2651280/Marvels_SpiderMan_2/","Abrir Steam")</f>
@@ -8209,16 +8209,16 @@
         <v>15</v>
       </c>
       <c r="D178">
-        <v>26428</v>
+        <v>26381</v>
       </c>
       <c r="E178">
         <v>109608</v>
       </c>
       <c r="F178">
-        <v>53428</v>
+        <v>53381</v>
       </c>
       <c r="G178">
-        <v>76936</v>
+        <v>76869</v>
       </c>
       <c r="H178">
         <v>27000</v>
@@ -8734,16 +8734,16 @@
         <v>15</v>
       </c>
       <c r="D190">
-        <v>29831</v>
+        <v>29768</v>
       </c>
       <c r="E190">
         <v>95904</v>
       </c>
       <c r="F190">
-        <v>56831</v>
+        <v>56768</v>
       </c>
       <c r="G190">
-        <v>81837</v>
+        <v>81746</v>
       </c>
       <c r="H190">
         <v>27000</v>
@@ -8823,16 +8823,16 @@
         <v>15</v>
       </c>
       <c r="D192">
-        <v>41944</v>
+        <v>41928</v>
       </c>
       <c r="E192">
         <v>123311</v>
       </c>
       <c r="F192">
-        <v>68944</v>
+        <v>68928</v>
       </c>
       <c r="G192">
-        <v>99279</v>
+        <v>99256</v>
       </c>
       <c r="H192">
         <v>27000</v>
@@ -9356,16 +9356,16 @@
         <v>15</v>
       </c>
       <c r="D204">
-        <v>29128</v>
+        <v>29035</v>
       </c>
       <c r="E204">
         <v>182692</v>
       </c>
       <c r="F204">
-        <v>56128</v>
+        <v>56035</v>
       </c>
       <c r="G204">
-        <v>80824</v>
+        <v>80690</v>
       </c>
       <c r="H204">
         <v>27000</v>
@@ -10059,16 +10059,16 @@
         <v>15</v>
       </c>
       <c r="D220">
-        <v>59302</v>
+        <v>59287</v>
       </c>
       <c r="E220">
         <v>82220</v>
       </c>
       <c r="F220">
-        <v>74302</v>
+        <v>74287</v>
       </c>
       <c r="G220">
-        <v>106995</v>
+        <v>106973</v>
       </c>
       <c r="H220">
         <v>15000</v>
@@ -10149,19 +10149,19 @@
         <v>15</v>
       </c>
       <c r="D222">
-        <v>0</v>
+        <v>74491</v>
       </c>
       <c r="E222">
         <v>96836</v>
       </c>
       <c r="F222">
-        <v>0</v>
+        <v>89491</v>
       </c>
       <c r="G222">
-        <v>0</v>
+        <v>128867</v>
       </c>
       <c r="H222">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="I222" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/3357650/PRAGMATA/","Abrir Steam")</f>
@@ -10239,19 +10239,19 @@
         <v>15</v>
       </c>
       <c r="D224">
-        <v>16203</v>
+        <v>16578</v>
       </c>
       <c r="E224">
         <v>60276</v>
       </c>
       <c r="F224">
-        <v>39605</v>
+        <v>39755</v>
       </c>
       <c r="G224">
-        <v>57031</v>
+        <v>57247</v>
       </c>
       <c r="H224">
-        <v>23402</v>
+        <v>23177</v>
       </c>
       <c r="I224" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/1144200/Ready_or_Not/","Abrir Steam")</f>
@@ -10589,7 +10589,7 @@
         <v>15</v>
       </c>
       <c r="D232">
-        <v>9335</v>
+        <v>9382</v>
       </c>
       <c r="E232">
         <v>52986</v>
@@ -10601,7 +10601,7 @@
         <v>49918</v>
       </c>
       <c r="H232">
-        <v>25330</v>
+        <v>25283</v>
       </c>
       <c r="I232" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/883710/Resident_Evil_2/?curator_clanid=4777282","Abrir Steam")</f>
@@ -10764,19 +10764,19 @@
         <v>15</v>
       </c>
       <c r="D236">
-        <v>8351</v>
+        <v>0</v>
       </c>
       <c r="E236">
         <v>52986</v>
       </c>
       <c r="F236">
-        <v>34717</v>
+        <v>0</v>
       </c>
       <c r="G236">
-        <v>49992</v>
+        <v>0</v>
       </c>
       <c r="H236">
-        <v>26366</v>
+        <v>0</v>
       </c>
       <c r="I236" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/952060/Resident_Evil_3/?curator_clanid=4777282","Abrir Steam")</f>
@@ -11028,19 +11028,19 @@
         <v>15</v>
       </c>
       <c r="D242">
-        <v>34561</v>
+        <v>0</v>
       </c>
       <c r="E242">
         <v>71257</v>
       </c>
       <c r="F242">
-        <v>51890</v>
+        <v>0</v>
       </c>
       <c r="G242">
-        <v>74722</v>
+        <v>0</v>
       </c>
       <c r="H242">
-        <v>17329</v>
+        <v>0</v>
       </c>
       <c r="I242" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/1196590/Resident_Evil_Village/?l=spanish","Abrir Steam")</f>
@@ -11291,16 +11291,16 @@
         <v>15</v>
       </c>
       <c r="D248">
-        <v>60208</v>
+        <v>60161</v>
       </c>
       <c r="E248">
         <v>96836</v>
       </c>
       <c r="F248">
-        <v>75208</v>
+        <v>75161</v>
       </c>
       <c r="G248">
-        <v>108300</v>
+        <v>108232</v>
       </c>
       <c r="H248">
         <v>15000</v>
@@ -11558,16 +11558,16 @@
         <v>15</v>
       </c>
       <c r="D254">
-        <v>16750</v>
+        <v>16718</v>
       </c>
       <c r="E254">
         <v>71257</v>
       </c>
       <c r="F254">
-        <v>43750</v>
+        <v>43718</v>
       </c>
       <c r="G254">
-        <v>63000</v>
+        <v>62954</v>
       </c>
       <c r="H254">
         <v>27000</v>
@@ -12171,19 +12171,19 @@
         <v>15</v>
       </c>
       <c r="D268">
-        <v>36246</v>
+        <v>0</v>
       </c>
       <c r="E268">
         <v>60276</v>
       </c>
       <c r="F268">
-        <v>51246</v>
+        <v>0</v>
       </c>
       <c r="G268">
-        <v>73794</v>
+        <v>0</v>
       </c>
       <c r="H268">
-        <v>15000</v>
+        <v>0</v>
       </c>
       <c r="I268" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/2947440/SILENT_HILL_f/","Abrir Steam")</f>
@@ -12438,19 +12438,19 @@
         <v>15</v>
       </c>
       <c r="D274">
-        <v>21854</v>
+        <v>0</v>
       </c>
       <c r="E274">
         <v>127879</v>
       </c>
       <c r="F274">
-        <v>48854</v>
+        <v>0</v>
       </c>
       <c r="G274">
-        <v>70350</v>
+        <v>0</v>
       </c>
       <c r="H274">
-        <v>27000</v>
+        <v>0</v>
       </c>
       <c r="I274" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/1774580/STAR_WARS_Jedi_Survivor/?curator_clanid=4777282","Abrir Steam")</f>
@@ -12525,16 +12525,16 @@
         <v>15</v>
       </c>
       <c r="D276">
-        <v>151917</v>
+        <v>151729</v>
       </c>
       <c r="E276">
         <v>164421</v>
       </c>
       <c r="F276">
-        <v>166917</v>
+        <v>166729</v>
       </c>
       <c r="G276">
-        <v>240360</v>
+        <v>240090</v>
       </c>
       <c r="H276">
         <v>15000</v>
@@ -13668,16 +13668,16 @@
         <v>15</v>
       </c>
       <c r="D302">
-        <v>18498</v>
+        <v>18435</v>
       </c>
       <c r="E302">
         <v>91337</v>
       </c>
       <c r="F302">
-        <v>45498</v>
+        <v>45435</v>
       </c>
       <c r="G302">
-        <v>65517</v>
+        <v>65426</v>
       </c>
       <c r="H302">
         <v>27000</v>
@@ -13756,19 +13756,19 @@
         <v>15</v>
       </c>
       <c r="D304">
-        <v>44083</v>
+        <v>0</v>
       </c>
       <c r="E304">
         <v>109608</v>
       </c>
       <c r="F304">
-        <v>71083</v>
+        <v>0</v>
       </c>
       <c r="G304">
-        <v>102360</v>
+        <v>0</v>
       </c>
       <c r="H304">
-        <v>27000</v>
+        <v>0</v>
       </c>
       <c r="I304" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/2172010/Until_Dawn/?curator_clanid=4777282","Abrir Steam")</f>
@@ -13844,16 +13844,16 @@
         <v>15</v>
       </c>
       <c r="D306">
-        <v>24601</v>
+        <v>24476</v>
       </c>
       <c r="E306">
         <v>109608</v>
       </c>
       <c r="F306">
-        <v>51601</v>
+        <v>51476</v>
       </c>
       <c r="G306">
-        <v>74305</v>
+        <v>74125</v>
       </c>
       <c r="H306">
         <v>27000</v>
@@ -14020,19 +14020,19 @@
         <v>15</v>
       </c>
       <c r="D310">
-        <v>71275</v>
+        <v>0</v>
       </c>
       <c r="E310">
         <v>127879</v>
       </c>
       <c r="F310">
-        <v>92055</v>
+        <v>0</v>
       </c>
       <c r="G310">
-        <v>132559</v>
+        <v>0</v>
       </c>
       <c r="H310">
-        <v>20780</v>
+        <v>0</v>
       </c>
       <c r="I310" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/3717070/WWE_2K26/","Abrir Steam")</f>

</xml_diff>